<commit_message>
Data wrangling - progress diary: documentation notes
Adding documentation notes to the measurement filtering tests.
</commit_message>
<xml_diff>
--- a/genomics_dir/outputs/comparative_tables/onminbus_kw_1st_genomics_4Mar26.xlsx
+++ b/genomics_dir/outputs/comparative_tables/onminbus_kw_1st_genomics_4Mar26.xlsx
@@ -1981,7 +1981,7 @@
       </c>
       <c r="I2" s="21"/>
     </row>
-    <row r="3" spans="1:9" ht="13.5" hidden="1">
+    <row r="3" spans="1:9" hidden="1">
       <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>372.07805625510758</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="13.5" hidden="1">
+    <row r="4" spans="1:9" hidden="1">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -2207,7 +2207,7 @@
         <v>92.516281185406655</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="13.5" hidden="1">
+    <row r="11" spans="1:9" hidden="1">
       <c r="A11" s="7" t="s">
         <v>53</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>19.217608665595851</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="13.5" hidden="1">
+    <row r="12" spans="1:9" hidden="1">
       <c r="A12" s="7" t="s">
         <v>59</v>
       </c>
@@ -2259,7 +2259,7 @@
       <c r="H12" s="3"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="13.5" hidden="1">
+    <row r="13" spans="1:9" hidden="1">
       <c r="A13" s="7" t="s">
         <v>61</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>43.198845682827027</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="13.5" hidden="1">
+    <row r="14" spans="1:9" hidden="1">
       <c r="A14" s="7" t="s">
         <v>67</v>
       </c>
@@ -2317,7 +2317,7 @@
         <v>5.6626027280000164</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="13.5" hidden="1">
+    <row r="15" spans="1:9" hidden="1">
       <c r="A15" s="7" t="s">
         <v>73</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>8.5495774815371615</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="13.5" hidden="1">
+    <row r="18" spans="1:9" hidden="1">
       <c r="A18" s="7" t="s">
         <v>89</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>95.532355214762859</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" hidden="1">
       <c r="A36" s="7" t="s">
         <v>192</v>
       </c>
@@ -2955,7 +2955,7 @@
         <v>182.47334665703349</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" hidden="1">
       <c r="A37" s="7" t="s">
         <v>197</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>67.755893649389392</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" hidden="1">
       <c r="A38" s="7" t="s">
         <v>203</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>71.095383874289936</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" hidden="1">
       <c r="A42" s="7" t="s">
         <v>227</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>188.2247569977207</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" hidden="1">
       <c r="A43" s="7" t="s">
         <v>233</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>34.915276137491091</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" hidden="1">
       <c r="A44" s="7" t="s">
         <v>239</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>37.135098528985218</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" hidden="1">
       <c r="A48" s="7" t="s">
         <v>263</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>208.00653187201041</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" hidden="1">
       <c r="A49" s="7" t="s">
         <v>269</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>11.997987059694699</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" hidden="1">
       <c r="A50" s="7" t="s">
         <v>275</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>14.38185422109081</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="13.5" hidden="1">
+    <row r="57" spans="1:9" hidden="1">
       <c r="A57" s="7" t="s">
         <v>317</v>
       </c>
@@ -3564,7 +3564,7 @@
         <v>8.6740950067151967</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="13.5" hidden="1">
+    <row r="58" spans="1:9" hidden="1">
       <c r="A58" s="7" t="s">
         <v>323</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>8.945114153211188</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="13.5" hidden="1">
+    <row r="59" spans="1:9" hidden="1">
       <c r="A59" s="7" t="s">
         <v>329</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>10.799578913084989</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="13.5" hidden="1">
+    <row r="60" spans="1:9" hidden="1">
       <c r="A60" s="7" t="s">
         <v>335</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>147.59442096849489</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="13.5" hidden="1">
+    <row r="61" spans="1:9" hidden="1">
       <c r="A61" s="7" t="s">
         <v>341</v>
       </c>
@@ -3680,7 +3680,7 @@
         <v>1.646684630415775</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="13.5" hidden="1">
+    <row r="62" spans="1:9" hidden="1">
       <c r="A62" s="7" t="s">
         <v>347</v>
       </c>
@@ -3709,7 +3709,7 @@
         <v>1.805223828200164</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="13.5" hidden="1">
+    <row r="63" spans="1:9" hidden="1">
       <c r="A63" s="7" t="s">
         <v>353</v>
       </c>
@@ -3738,7 +3738,7 @@
         <v>1.4489901329389021</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="13.5" hidden="1">
+    <row r="64" spans="1:9" hidden="1">
       <c r="A64" s="7" t="s">
         <v>359</v>
       </c>
@@ -3767,7 +3767,7 @@
         <v>1.337577348716313</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="13.5" hidden="1">
+    <row r="65" spans="1:9" hidden="1">
       <c r="A65" s="7" t="s">
         <v>365</v>
       </c>
@@ -3796,7 +3796,7 @@
         <v>1.751147266969072</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="13.5" hidden="1">
+    <row r="66" spans="1:9" hidden="1">
       <c r="A66" s="7" t="s">
         <v>371</v>
       </c>
@@ -3825,7 +3825,7 @@
         <v>164.8018165954494</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="13.5" hidden="1">
+    <row r="67" spans="1:9" hidden="1">
       <c r="A67" s="7" t="s">
         <v>377</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>3.9750873131594342</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="13.5" hidden="1">
+    <row r="68" spans="1:9" hidden="1">
       <c r="A68" s="7" t="s">
         <v>383</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>1.5611460963432851</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="13.5" hidden="1">
+    <row r="69" spans="1:9" hidden="1">
       <c r="A69" s="7" t="s">
         <v>389</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>3.391603522369036</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="13.5" hidden="1">
+    <row r="70" spans="1:9" hidden="1">
       <c r="A70" s="7" t="s">
         <v>395</v>
       </c>
@@ -3941,7 +3941,7 @@
         <v>4.5647456063094314</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="13.5" hidden="1">
+    <row r="71" spans="1:9" hidden="1">
       <c r="A71" s="7" t="s">
         <v>401</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>4.8150413919639377</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="13.5" hidden="1">
+    <row r="72" spans="1:9" hidden="1">
       <c r="A72" s="7" t="s">
         <v>407</v>
       </c>
@@ -3999,7 +3999,7 @@
         <v>219.56629546221461</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="13.5" hidden="1">
+    <row r="73" spans="1:9" hidden="1">
       <c r="A73" s="7" t="s">
         <v>412</v>
       </c>

</xml_diff>